<commit_message>
updated docs until June 11th
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD4B2B8E-CA6A-46B4-9309-B2AFE6D7B97B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FCA194-27D1-4A2B-A17F-DA757F3DE095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20655" yWindow="3675" windowWidth="19185" windowHeight="11265" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -263,6 +263,18 @@
   </si>
   <si>
     <t>O&amp;M saas repo</t>
+  </si>
+  <si>
+    <t>https://infoblox.net.rewe.intranet/ui/signin</t>
+  </si>
+  <si>
+    <t>InfoBlox</t>
+  </si>
+  <si>
+    <t>https://streaming.vault.rewe.cloud/ui/vault/secrets/secret/kv/list/team_seven/infoblox/</t>
+  </si>
+  <si>
+    <t>InfoBlox/T7/Vault</t>
   </si>
 </sst>
 </file>
@@ -436,8 +448,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}" name="Table3" displayName="Table3" ref="A3:C16" totalsRowShown="0">
-  <autoFilter ref="A3:C16" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}" name="Table3" displayName="Table3" ref="A3:C18" totalsRowShown="0">
+  <autoFilter ref="A3:C18" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{92DEE286-5F23-49AE-A993-EE800877A5EE}" name="Title"/>
     <tableColumn id="2" xr3:uid="{16826D26-E8CF-4027-A8E6-28B0A1A1041D}" name="URL" dataCellStyle="Hyperlink"/>
@@ -764,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51094AFD-03E5-4E2E-A855-873D3CEE7610}">
-  <dimension ref="A3:C16"/>
+  <dimension ref="A3:C18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -891,6 +903,22 @@
       </c>
       <c r="B16" s="3" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -908,11 +936,13 @@
     <hyperlink ref="B5" r:id="rId11" xr:uid="{997FA379-5083-4A11-A6D1-809BA5407CED}"/>
     <hyperlink ref="B15" r:id="rId12" xr:uid="{3F6F8243-51FF-46D2-9E1F-36AA9EE212C8}"/>
     <hyperlink ref="B16" r:id="rId13" xr:uid="{F8618F85-9977-4563-AF67-F876A4278094}"/>
+    <hyperlink ref="B17" r:id="rId14" xr:uid="{EE19D4E7-BA71-4CDD-8A0C-E76879C0114D}"/>
+    <hyperlink ref="B18" r:id="rId15" xr:uid="{348BA626-AC2D-468D-813D-6C20585F4A4A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId14"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
   <tableParts count="1">
-    <tablePart r:id="rId15"/>
+    <tablePart r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Latest notes updates as of July 29
</commit_message>
<xml_diff>
--- a/SEVEN_Kakfa_Links.xlsx
+++ b/SEVEN_Kakfa_Links.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A233C1F\Documents\Docs&amp;Misc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FCA194-27D1-4A2B-A17F-DA757F3DE095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A1A9E21-24D4-49D7-B8D2-E4AE7B8D550A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
+    <workbookView xWindow="-28920" yWindow="1050" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{9D751822-9D83-4D60-B2B6-9E7CF2D78AD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Links" sheetId="1" r:id="rId1"/>
     <sheet name="Kafka Self Service" sheetId="2" r:id="rId2"/>
     <sheet name="RTP" sheetId="3" r:id="rId3"/>
-    <sheet name="Change control" sheetId="4" r:id="rId4"/>
+    <sheet name="OnCall" sheetId="5" r:id="rId4"/>
+    <sheet name="Change control" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="52">
   <si>
     <t>https://rewe.atlassian.net/wiki/spaces/TITISEVEN/pages/1134952479/System+overview+Kafka+Clusters+managed+by+Team+SEVEN</t>
   </si>
@@ -275,6 +277,12 @@
   </si>
   <si>
     <t>InfoBlox/T7/Vault</t>
+  </si>
+  <si>
+    <t>Streaming &amp; Eventing Platform</t>
+  </si>
+  <si>
+    <t>https://console.prod.kafka.rewe.cloud/console/bd-prd/home</t>
   </si>
 </sst>
 </file>
@@ -448,8 +456,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}" name="Table3" displayName="Table3" ref="A3:C18" totalsRowShown="0">
-  <autoFilter ref="A3:C18" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}" name="Table3" displayName="Table3" ref="A3:C19" totalsRowShown="0">
+  <autoFilter ref="A3:C19" xr:uid="{4FEFBF19-B0BB-4FF9-82D1-B22F0F681040}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{92DEE286-5F23-49AE-A993-EE800877A5EE}" name="Title"/>
     <tableColumn id="2" xr3:uid="{16826D26-E8CF-4027-A8E6-28B0A1A1041D}" name="URL" dataCellStyle="Hyperlink"/>
@@ -776,7 +784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51094AFD-03E5-4E2E-A855-873D3CEE7610}">
-  <dimension ref="A3:C18"/>
+  <dimension ref="A3:C19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19.54296875" customWidth="1"/>
@@ -919,6 +927,11 @@
       </c>
       <c r="B18" s="3" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B19" s="3" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -938,11 +951,12 @@
     <hyperlink ref="B16" r:id="rId13" xr:uid="{F8618F85-9977-4563-AF67-F876A4278094}"/>
     <hyperlink ref="B17" r:id="rId14" xr:uid="{EE19D4E7-BA71-4CDD-8A0C-E76879C0114D}"/>
     <hyperlink ref="B18" r:id="rId15" xr:uid="{348BA626-AC2D-468D-813D-6C20585F4A4A}"/>
+    <hyperlink ref="B19" r:id="rId16" xr:uid="{FA5A231A-441F-443A-9A4C-E4587EB0FC97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId16"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
   <tableParts count="1">
-    <tablePart r:id="rId17"/>
+    <tablePart r:id="rId18"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1038,6 +1052,24 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B176F9-BD63-46E4-9E06-792BB9828535}">
+  <dimension ref="A3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" display="https://risnet.sharepoint.com/:f:/r/sites/NearshoreSpain/Freigegebene Dokumente/General/08_Finance %26 Accounting/Input Payroll/2026/2026 On-Call Duty Reports/Streaming %26 Eventing Platform?csf=1&amp;web=1&amp;e=zRpVoH" xr:uid="{C00ECCC9-D3DE-4B55-81FC-464EE11CCF21}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF4F27D-A951-431B-81D5-DDDFCFE35034}">
   <dimension ref="O11:O13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>